<commit_message>
Lots of changes to facilitate state Inventory. National data for 1990-2023 is in temporaru_national_inv_data.csv; this is a short-term measure until full inventory pipeline is complete. Also fixed a bunch of weird unit-conversion issues in state calcs.
</commit_message>
<xml_diff>
--- a/data/international_bunker_fuels.xlsx
+++ b/data/international_bunker_fuels.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DB154AC-31A3-4F66-93D5-838312B96F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{6DB154AC-31A3-4F66-93D5-838312B96F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF769A53-DD68-43E5-B94D-A9698BB80AFD}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0D0EB5BF-8D36-4958-8217-247236FD9C13}"/>
+    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{0D0EB5BF-8D36-4958-8217-247236FD9C13}"/>
   </bookViews>
   <sheets>
     <sheet name="ibf" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -54,21 +54,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.00_)"/>
-  </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -407,10 +399,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F26182C8-B79B-4DC7-B7F8-093E556E80AF}">
-  <dimension ref="A1:AH4"/>
+  <dimension ref="A1:AI4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,8 +505,11 @@
       <c r="AH1">
         <v>2022</v>
       </c>
+      <c r="AI1">
+        <v>2023</v>
+      </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -617,8 +612,11 @@
       <c r="AH2">
         <v>945.55835987107741</v>
       </c>
+      <c r="AI2">
+        <v>943.89917779577081</v>
+      </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -721,8 +719,11 @@
       <c r="AH3">
         <v>325.17659121999998</v>
       </c>
+      <c r="AI3">
+        <v>301.79992203500001</v>
+      </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -824,6 +825,9 @@
       </c>
       <c r="AH4">
         <v>96.810063081760362</v>
+      </c>
+      <c r="AI4">
+        <v>94.033723713601191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>